<commit_message>
Anonymize coder identities (Coder 1/2/3) in human-coding data files
</commit_message>
<xml_diff>
--- a/data/human_coding_κ試打_20260620.xlsx
+++ b/data/human_coding_κ試打_20260620.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KEY（解盲）" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月島評分" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地理老師評分" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第三人評分（限事實糾正格）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coder 1評分" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coder 2評分" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coder 3評分（限事實糾正格）" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="κ 一致度" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
@@ -2177,6 +2177,57 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
@@ -11020,17 +11071,17 @@
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
-          <t>〔格7暫存〕第三人ID</t>
+          <t>〔格7暫存〕Coder 3ID</t>
         </is>
       </c>
       <c r="I1" s="7" t="inlineStr">
         <is>
-          <t>第三人格7</t>
+          <t>Coder 3格7</t>
         </is>
       </c>
       <c r="J1" s="7" t="inlineStr">
         <is>
-          <t>地理老師格7(對同ID)</t>
+          <t>Coder 2格7(對同ID)</t>
         </is>
       </c>
     </row>
@@ -11046,11 +11097,11 @@
         </is>
       </c>
       <c r="C2" s="8">
-        <f>SUMPRODUCT(('月島評分'!C2:C101&lt;&gt;"")*('地理老師評分'!C2:C101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!C2:C101&lt;&gt;"")*('Coder 2評分'!C2:C101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D2" s="8">
-        <f>SUMPRODUCT(('月島評分'!C2:C101='地理老師評分'!C2:C101)*('月島評分'!C2:C101&lt;&gt;"")*('地理老師評分'!C2:C101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!C2:C101='Coder 2評分'!C2:C101)*('Coder 1評分'!C2:C101&lt;&gt;"")*('Coder 2評分'!C2:C101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E2" s="9">
@@ -11062,15 +11113,15 @@
         <v/>
       </c>
       <c r="H2">
-        <f>'第三人評分（限事實糾正格）'!A2</f>
+        <f>'Coder 3評分（限事實糾正格）'!A2</f>
         <v/>
       </c>
       <c r="I2">
-        <f>'第三人評分（限事實糾正格）'!C2</f>
+        <f>'Coder 3評分（限事實糾正格）'!C2</f>
         <v/>
       </c>
       <c r="J2">
-        <f>IFERROR(XLOOKUP(H2,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H2,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11086,11 +11137,11 @@
         </is>
       </c>
       <c r="C3" s="8">
-        <f>SUMPRODUCT(('月島評分'!E2:E101&lt;&gt;"")*('地理老師評分'!E2:E101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!E2:E101&lt;&gt;"")*('Coder 2評分'!E2:E101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D3" s="8">
-        <f>SUMPRODUCT(('月島評分'!E2:E101='地理老師評分'!E2:E101)*('月島評分'!E2:E101&lt;&gt;"")*('地理老師評分'!E2:E101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!E2:E101='Coder 2評分'!E2:E101)*('Coder 1評分'!E2:E101&lt;&gt;"")*('Coder 2評分'!E2:E101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E3" s="9">
@@ -11102,15 +11153,15 @@
         <v/>
       </c>
       <c r="H3">
-        <f>'第三人評分（限事實糾正格）'!A3</f>
+        <f>'Coder 3評分（限事實糾正格）'!A3</f>
         <v/>
       </c>
       <c r="I3">
-        <f>'第三人評分（限事實糾正格）'!C3</f>
+        <f>'Coder 3評分（限事實糾正格）'!C3</f>
         <v/>
       </c>
       <c r="J3">
-        <f>IFERROR(XLOOKUP(H3,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H3,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11126,11 +11177,11 @@
         </is>
       </c>
       <c r="C4" s="8">
-        <f>SUMPRODUCT(('月島評分'!G2:G101&lt;&gt;"")*('地理老師評分'!G2:G101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!G2:G101&lt;&gt;"")*('Coder 2評分'!G2:G101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D4" s="8">
-        <f>SUMPRODUCT(('月島評分'!G2:G101='地理老師評分'!G2:G101)*('月島評分'!G2:G101&lt;&gt;"")*('地理老師評分'!G2:G101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!G2:G101='Coder 2評分'!G2:G101)*('Coder 1評分'!G2:G101&lt;&gt;"")*('Coder 2評分'!G2:G101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E4" s="9">
@@ -11142,15 +11193,15 @@
         <v/>
       </c>
       <c r="H4">
-        <f>'第三人評分（限事實糾正格）'!A4</f>
+        <f>'Coder 3評分（限事實糾正格）'!A4</f>
         <v/>
       </c>
       <c r="I4">
-        <f>'第三人評分（限事實糾正格）'!C4</f>
+        <f>'Coder 3評分（限事實糾正格）'!C4</f>
         <v/>
       </c>
       <c r="J4">
-        <f>IFERROR(XLOOKUP(H4,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H4,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11166,11 +11217,11 @@
         </is>
       </c>
       <c r="C5" s="8">
-        <f>SUMPRODUCT(('月島評分'!I2:I101&lt;&gt;"")*('地理老師評分'!I2:I101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!I2:I101&lt;&gt;"")*('Coder 2評分'!I2:I101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D5" s="8">
-        <f>SUMPRODUCT(('月島評分'!I2:I101='地理老師評分'!I2:I101)*('月島評分'!I2:I101&lt;&gt;"")*('地理老師評分'!I2:I101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!I2:I101='Coder 2評分'!I2:I101)*('Coder 1評分'!I2:I101&lt;&gt;"")*('Coder 2評分'!I2:I101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E5" s="9">
@@ -11182,15 +11233,15 @@
         <v/>
       </c>
       <c r="H5">
-        <f>'第三人評分（限事實糾正格）'!A5</f>
+        <f>'Coder 3評分（限事實糾正格）'!A5</f>
         <v/>
       </c>
       <c r="I5">
-        <f>'第三人評分（限事實糾正格）'!C5</f>
+        <f>'Coder 3評分（限事實糾正格）'!C5</f>
         <v/>
       </c>
       <c r="J5">
-        <f>IFERROR(XLOOKUP(H5,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H5,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11206,11 +11257,11 @@
         </is>
       </c>
       <c r="C6">
-        <f>SUMPRODUCT(('月島評分'!K2:K101&lt;&gt;"")*('地理老師評分'!K2:K101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!K2:K101&lt;&gt;"")*('Coder 2評分'!K2:K101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT(('月島評分'!K2:K101='地理老師評分'!K2:K101)*('月島評分'!K2:K101&lt;&gt;"")*('地理老師評分'!K2:K101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!K2:K101='Coder 2評分'!K2:K101)*('Coder 1評分'!K2:K101&lt;&gt;"")*('Coder 2評分'!K2:K101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E6" s="10">
@@ -11222,15 +11273,15 @@
         <v/>
       </c>
       <c r="H6">
-        <f>'第三人評分（限事實糾正格）'!A6</f>
+        <f>'Coder 3評分（限事實糾正格）'!A6</f>
         <v/>
       </c>
       <c r="I6">
-        <f>'第三人評分（限事實糾正格）'!C6</f>
+        <f>'Coder 3評分（限事實糾正格）'!C6</f>
         <v/>
       </c>
       <c r="J6">
-        <f>IFERROR(XLOOKUP(H6,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H6,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11246,11 +11297,11 @@
         </is>
       </c>
       <c r="C7">
-        <f>SUMPRODUCT(('月島評分'!M2:M101&lt;&gt;"")*('地理老師評分'!M2:M101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!M2:M101&lt;&gt;"")*('Coder 2評分'!M2:M101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT(('月島評分'!M2:M101='地理老師評分'!M2:M101)*('月島評分'!M2:M101&lt;&gt;"")*('地理老師評分'!M2:M101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!M2:M101='Coder 2評分'!M2:M101)*('Coder 1評分'!M2:M101&lt;&gt;"")*('Coder 2評分'!M2:M101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E7" s="10">
@@ -11262,15 +11313,15 @@
         <v/>
       </c>
       <c r="H7">
-        <f>'第三人評分（限事實糾正格）'!A7</f>
+        <f>'Coder 3評分（限事實糾正格）'!A7</f>
         <v/>
       </c>
       <c r="I7">
-        <f>'第三人評分（限事實糾正格）'!C7</f>
+        <f>'Coder 3評分（限事實糾正格）'!C7</f>
         <v/>
       </c>
       <c r="J7">
-        <f>IFERROR(XLOOKUP(H7,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H7,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11286,11 +11337,11 @@
         </is>
       </c>
       <c r="C8">
-        <f>SUMPRODUCT(('月島評分'!O2:O101&lt;&gt;"")*('地理老師評分'!O2:O101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!O2:O101&lt;&gt;"")*('Coder 2評分'!O2:O101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT(('月島評分'!O2:O101='地理老師評分'!O2:O101)*('月島評分'!O2:O101&lt;&gt;"")*('地理老師評分'!O2:O101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!O2:O101='Coder 2評分'!O2:O101)*('Coder 1評分'!O2:O101&lt;&gt;"")*('Coder 2評分'!O2:O101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E8" s="10">
@@ -11302,15 +11353,15 @@
         <v/>
       </c>
       <c r="H8">
-        <f>'第三人評分（限事實糾正格）'!A8</f>
+        <f>'Coder 3評分（限事實糾正格）'!A8</f>
         <v/>
       </c>
       <c r="I8">
-        <f>'第三人評分（限事實糾正格）'!C8</f>
+        <f>'Coder 3評分（限事實糾正格）'!C8</f>
         <v/>
       </c>
       <c r="J8">
-        <f>IFERROR(XLOOKUP(H8,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H8,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11342,15 +11393,15 @@
         <v/>
       </c>
       <c r="H9">
-        <f>'第三人評分（限事實糾正格）'!A9</f>
+        <f>'Coder 3評分（限事實糾正格）'!A9</f>
         <v/>
       </c>
       <c r="I9">
-        <f>'第三人評分（限事實糾正格）'!C9</f>
+        <f>'Coder 3評分（限事實糾正格）'!C9</f>
         <v/>
       </c>
       <c r="J9">
-        <f>IFERROR(XLOOKUP(H9,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H9,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11366,11 +11417,11 @@
         </is>
       </c>
       <c r="C10">
-        <f>SUMPRODUCT(('月島評分'!T2:T101&lt;&gt;"")*('地理老師評分'!T2:T101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!T2:T101&lt;&gt;"")*('Coder 2評分'!T2:T101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D10">
-        <f>SUMPRODUCT(('月島評分'!T2:T101='地理老師評分'!T2:T101)*('月島評分'!T2:T101&lt;&gt;"")*('地理老師評分'!T2:T101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!T2:T101='Coder 2評分'!T2:T101)*('Coder 1評分'!T2:T101&lt;&gt;"")*('Coder 2評分'!T2:T101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E10" s="10">
@@ -11382,15 +11433,15 @@
         <v/>
       </c>
       <c r="H10">
-        <f>'第三人評分（限事實糾正格）'!A10</f>
+        <f>'Coder 3評分（限事實糾正格）'!A10</f>
         <v/>
       </c>
       <c r="I10">
-        <f>'第三人評分（限事實糾正格）'!C10</f>
+        <f>'Coder 3評分（限事實糾正格）'!C10</f>
         <v/>
       </c>
       <c r="J10">
-        <f>IFERROR(XLOOKUP(H10,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H10,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11406,11 +11457,11 @@
         </is>
       </c>
       <c r="C11">
-        <f>SUMPRODUCT(('月島評分'!V2:V101&lt;&gt;"")*('地理老師評分'!V2:V101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!V2:V101&lt;&gt;"")*('Coder 2評分'!V2:V101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="D11">
-        <f>SUMPRODUCT(('月島評分'!V2:V101='地理老師評分'!V2:V101)*('月島評分'!V2:V101&lt;&gt;"")*('地理老師評分'!V2:V101&lt;&gt;""))</f>
+        <f>SUMPRODUCT(('Coder 1評分'!V2:V101='Coder 2評分'!V2:V101)*('Coder 1評分'!V2:V101&lt;&gt;"")*('Coder 2評分'!V2:V101&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="E11" s="10">
@@ -11422,29 +11473,29 @@
         <v/>
       </c>
       <c r="H11">
-        <f>'第三人評分（限事實糾正格）'!A11</f>
+        <f>'Coder 3評分（限事實糾正格）'!A11</f>
         <v/>
       </c>
       <c r="I11">
-        <f>'第三人評分（限事實糾正格）'!C11</f>
+        <f>'Coder 3評分（限事實糾正格）'!C11</f>
         <v/>
       </c>
       <c r="J11">
-        <f>IFERROR(XLOOKUP(H11,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H11,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="H12">
-        <f>'第三人評分（限事實糾正格）'!A12</f>
+        <f>'Coder 3評分（限事實糾正格）'!A12</f>
         <v/>
       </c>
       <c r="I12">
-        <f>'第三人評分（限事實糾正格）'!C12</f>
+        <f>'Coder 3評分（限事實糾正格）'!C12</f>
         <v/>
       </c>
       <c r="J12">
-        <f>IFERROR(XLOOKUP(H12,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H12,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11455,15 +11506,15 @@
         </is>
       </c>
       <c r="H13">
-        <f>'第三人評分（限事實糾正格）'!A13</f>
+        <f>'Coder 3評分（限事實糾正格）'!A13</f>
         <v/>
       </c>
       <c r="I13">
-        <f>'第三人評分（限事實糾正格）'!C13</f>
+        <f>'Coder 3評分（限事實糾正格）'!C13</f>
         <v/>
       </c>
       <c r="J13">
-        <f>IFERROR(XLOOKUP(H13,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H13,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11474,15 +11525,15 @@
         </is>
       </c>
       <c r="H14">
-        <f>'第三人評分（限事實糾正格）'!A14</f>
+        <f>'Coder 3評分（限事實糾正格）'!A14</f>
         <v/>
       </c>
       <c r="I14">
-        <f>'第三人評分（限事實糾正格）'!C14</f>
+        <f>'Coder 3評分（限事實糾正格）'!C14</f>
         <v/>
       </c>
       <c r="J14">
-        <f>IFERROR(XLOOKUP(H14,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H14,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11493,15 +11544,15 @@
         </is>
       </c>
       <c r="H15">
-        <f>'第三人評分（限事實糾正格）'!A15</f>
+        <f>'Coder 3評分（限事實糾正格）'!A15</f>
         <v/>
       </c>
       <c r="I15">
-        <f>'第三人評分（限事實糾正格）'!C15</f>
+        <f>'Coder 3評分（限事實糾正格）'!C15</f>
         <v/>
       </c>
       <c r="J15">
-        <f>IFERROR(XLOOKUP(H15,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H15,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11512,15 +11563,15 @@
         </is>
       </c>
       <c r="H16">
-        <f>'第三人評分（限事實糾正格）'!A16</f>
+        <f>'Coder 3評分（限事實糾正格）'!A16</f>
         <v/>
       </c>
       <c r="I16">
-        <f>'第三人評分（限事實糾正格）'!C16</f>
+        <f>'Coder 3評分（限事實糾正格）'!C16</f>
         <v/>
       </c>
       <c r="J16">
-        <f>IFERROR(XLOOKUP(H16,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H16,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11531,49 +11582,49 @@
         </is>
       </c>
       <c r="H17">
-        <f>'第三人評分（限事實糾正格）'!A17</f>
+        <f>'Coder 3評分（限事實糾正格）'!A17</f>
         <v/>
       </c>
       <c r="I17">
-        <f>'第三人評分（限事實糾正格）'!C17</f>
+        <f>'Coder 3評分（限事實糾正格）'!C17</f>
         <v/>
       </c>
       <c r="J17">
-        <f>IFERROR(XLOOKUP(H17,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H17,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>5. 格7 由第三人評，κ 算「地理老師 vs 第三人」（外審 Q6=A，避月島自評偏誤）；月島不評格7</t>
+          <t>5. 格7 由Coder 3評，κ 算「Coder 2 vs Coder 3」（外審 Q6=A，避Coder 1自評偏誤）；Coder 1不評格7</t>
         </is>
       </c>
       <c r="H18">
-        <f>'第三人評分（限事實糾正格）'!A18</f>
+        <f>'Coder 3評分（限事實糾正格）'!A18</f>
         <v/>
       </c>
       <c r="I18">
-        <f>'第三人評分（限事實糾正格）'!C18</f>
+        <f>'Coder 3評分（限事實糾正格）'!C18</f>
         <v/>
       </c>
       <c r="J18">
-        <f>IFERROR(XLOOKUP(H18,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H18,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr"/>
       <c r="H19">
-        <f>'第三人評分（限事實糾正格）'!A19</f>
+        <f>'Coder 3評分（限事實糾正格）'!A19</f>
         <v/>
       </c>
       <c r="I19">
-        <f>'第三人評分（限事實糾正格）'!C19</f>
+        <f>'Coder 3評分（限事實糾正格）'!C19</f>
         <v/>
       </c>
       <c r="J19">
-        <f>IFERROR(XLOOKUP(H19,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H19,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11584,15 +11635,15 @@
         </is>
       </c>
       <c r="H20">
-        <f>'第三人評分（限事實糾正格）'!A20</f>
+        <f>'Coder 3評分（限事實糾正格）'!A20</f>
         <v/>
       </c>
       <c r="I20">
-        <f>'第三人評分（限事實糾正格）'!C20</f>
+        <f>'Coder 3評分（限事實糾正格）'!C20</f>
         <v/>
       </c>
       <c r="J20">
-        <f>IFERROR(XLOOKUP(H20,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H20,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11603,30 +11654,30 @@
         </is>
       </c>
       <c r="H21">
-        <f>'第三人評分（限事實糾正格）'!A21</f>
+        <f>'Coder 3評分（限事實糾正格）'!A21</f>
         <v/>
       </c>
       <c r="I21">
-        <f>'第三人評分（限事實糾正格）'!C21</f>
+        <f>'Coder 3評分（限事實糾正格）'!C21</f>
         <v/>
       </c>
       <c r="J21">
-        <f>IFERROR(XLOOKUP(H21,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H21,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr"/>
       <c r="H22">
-        <f>'第三人評分（限事實糾正格）'!A22</f>
+        <f>'Coder 3評分（限事實糾正格）'!A22</f>
         <v/>
       </c>
       <c r="I22">
-        <f>'第三人評分（限事實糾正格）'!C22</f>
+        <f>'Coder 3評分（限事實糾正格）'!C22</f>
         <v/>
       </c>
       <c r="J22">
-        <f>IFERROR(XLOOKUP(H22,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H22,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11637,15 +11688,15 @@
         </is>
       </c>
       <c r="H23">
-        <f>'第三人評分（限事實糾正格）'!A23</f>
+        <f>'Coder 3評分（限事實糾正格）'!A23</f>
         <v/>
       </c>
       <c r="I23">
-        <f>'第三人評分（限事實糾正格）'!C23</f>
+        <f>'Coder 3評分（限事實糾正格）'!C23</f>
         <v/>
       </c>
       <c r="J23">
-        <f>IFERROR(XLOOKUP(H23,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H23,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11656,15 +11707,15 @@
         </is>
       </c>
       <c r="H24">
-        <f>'第三人評分（限事實糾正格）'!A24</f>
+        <f>'Coder 3評分（限事實糾正格）'!A24</f>
         <v/>
       </c>
       <c r="I24">
-        <f>'第三人評分（限事實糾正格）'!C24</f>
+        <f>'Coder 3評分（限事實糾正格）'!C24</f>
         <v/>
       </c>
       <c r="J24">
-        <f>IFERROR(XLOOKUP(H24,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H24,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11675,15 +11726,15 @@
         </is>
       </c>
       <c r="H25">
-        <f>'第三人評分（限事實糾正格）'!A25</f>
+        <f>'Coder 3評分（限事實糾正格）'!A25</f>
         <v/>
       </c>
       <c r="I25">
-        <f>'第三人評分（限事實糾正格）'!C25</f>
+        <f>'Coder 3評分（限事實糾正格）'!C25</f>
         <v/>
       </c>
       <c r="J25">
-        <f>IFERROR(XLOOKUP(H25,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H25,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11694,15 +11745,15 @@
         </is>
       </c>
       <c r="H26">
-        <f>'第三人評分（限事實糾正格）'!A26</f>
+        <f>'Coder 3評分（限事實糾正格）'!A26</f>
         <v/>
       </c>
       <c r="I26">
-        <f>'第三人評分（限事實糾正格）'!C26</f>
+        <f>'Coder 3評分（限事實糾正格）'!C26</f>
         <v/>
       </c>
       <c r="J26">
-        <f>IFERROR(XLOOKUP(H26,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H26,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11713,15 +11764,15 @@
         </is>
       </c>
       <c r="H27">
-        <f>'第三人評分（限事實糾正格）'!A27</f>
+        <f>'Coder 3評分（限事實糾正格）'!A27</f>
         <v/>
       </c>
       <c r="I27">
-        <f>'第三人評分（限事實糾正格）'!C27</f>
+        <f>'Coder 3評分（限事實糾正格）'!C27</f>
         <v/>
       </c>
       <c r="J27">
-        <f>IFERROR(XLOOKUP(H27,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H27,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11732,15 +11783,15 @@
         </is>
       </c>
       <c r="H28">
-        <f>'第三人評分（限事實糾正格）'!A28</f>
+        <f>'Coder 3評分（限事實糾正格）'!A28</f>
         <v/>
       </c>
       <c r="I28">
-        <f>'第三人評分（限事實糾正格）'!C28</f>
+        <f>'Coder 3評分（限事實糾正格）'!C28</f>
         <v/>
       </c>
       <c r="J28">
-        <f>IFERROR(XLOOKUP(H28,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H28,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
@@ -11751,1023 +11802,1023 @@
         </is>
       </c>
       <c r="H29">
-        <f>'第三人評分（限事實糾正格）'!A29</f>
+        <f>'Coder 3評分（限事實糾正格）'!A29</f>
         <v/>
       </c>
       <c r="I29">
-        <f>'第三人評分（限事實糾正格）'!C29</f>
+        <f>'Coder 3評分（限事實糾正格）'!C29</f>
         <v/>
       </c>
       <c r="J29">
-        <f>IFERROR(XLOOKUP(H29,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H29,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="H30">
-        <f>'第三人評分（限事實糾正格）'!A30</f>
+        <f>'Coder 3評分（限事實糾正格）'!A30</f>
         <v/>
       </c>
       <c r="I30">
-        <f>'第三人評分（限事實糾正格）'!C30</f>
+        <f>'Coder 3評分（限事實糾正格）'!C30</f>
         <v/>
       </c>
       <c r="J30">
-        <f>IFERROR(XLOOKUP(H30,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H30,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="H31">
-        <f>'第三人評分（限事實糾正格）'!A31</f>
+        <f>'Coder 3評分（限事實糾正格）'!A31</f>
         <v/>
       </c>
       <c r="I31">
-        <f>'第三人評分（限事實糾正格）'!C31</f>
+        <f>'Coder 3評分（限事實糾正格）'!C31</f>
         <v/>
       </c>
       <c r="J31">
-        <f>IFERROR(XLOOKUP(H31,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H31,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="H32">
-        <f>'第三人評分（限事實糾正格）'!A32</f>
+        <f>'Coder 3評分（限事實糾正格）'!A32</f>
         <v/>
       </c>
       <c r="I32">
-        <f>'第三人評分（限事實糾正格）'!C32</f>
+        <f>'Coder 3評分（限事實糾正格）'!C32</f>
         <v/>
       </c>
       <c r="J32">
-        <f>IFERROR(XLOOKUP(H32,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H32,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="H33">
-        <f>'第三人評分（限事實糾正格）'!A33</f>
+        <f>'Coder 3評分（限事實糾正格）'!A33</f>
         <v/>
       </c>
       <c r="I33">
-        <f>'第三人評分（限事實糾正格）'!C33</f>
+        <f>'Coder 3評分（限事實糾正格）'!C33</f>
         <v/>
       </c>
       <c r="J33">
-        <f>IFERROR(XLOOKUP(H33,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H33,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="H34">
-        <f>'第三人評分（限事實糾正格）'!A34</f>
+        <f>'Coder 3評分（限事實糾正格）'!A34</f>
         <v/>
       </c>
       <c r="I34">
-        <f>'第三人評分（限事實糾正格）'!C34</f>
+        <f>'Coder 3評分（限事實糾正格）'!C34</f>
         <v/>
       </c>
       <c r="J34">
-        <f>IFERROR(XLOOKUP(H34,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H34,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="H35">
-        <f>'第三人評分（限事實糾正格）'!A35</f>
+        <f>'Coder 3評分（限事實糾正格）'!A35</f>
         <v/>
       </c>
       <c r="I35">
-        <f>'第三人評分（限事實糾正格）'!C35</f>
+        <f>'Coder 3評分（限事實糾正格）'!C35</f>
         <v/>
       </c>
       <c r="J35">
-        <f>IFERROR(XLOOKUP(H35,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H35,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="H36">
-        <f>'第三人評分（限事實糾正格）'!A36</f>
+        <f>'Coder 3評分（限事實糾正格）'!A36</f>
         <v/>
       </c>
       <c r="I36">
-        <f>'第三人評分（限事實糾正格）'!C36</f>
+        <f>'Coder 3評分（限事實糾正格）'!C36</f>
         <v/>
       </c>
       <c r="J36">
-        <f>IFERROR(XLOOKUP(H36,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H36,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="H37">
-        <f>'第三人評分（限事實糾正格）'!A37</f>
+        <f>'Coder 3評分（限事實糾正格）'!A37</f>
         <v/>
       </c>
       <c r="I37">
-        <f>'第三人評分（限事實糾正格）'!C37</f>
+        <f>'Coder 3評分（限事實糾正格）'!C37</f>
         <v/>
       </c>
       <c r="J37">
-        <f>IFERROR(XLOOKUP(H37,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H37,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="H38">
-        <f>'第三人評分（限事實糾正格）'!A38</f>
+        <f>'Coder 3評分（限事實糾正格）'!A38</f>
         <v/>
       </c>
       <c r="I38">
-        <f>'第三人評分（限事實糾正格）'!C38</f>
+        <f>'Coder 3評分（限事實糾正格）'!C38</f>
         <v/>
       </c>
       <c r="J38">
-        <f>IFERROR(XLOOKUP(H38,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H38,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="H39">
-        <f>'第三人評分（限事實糾正格）'!A39</f>
+        <f>'Coder 3評分（限事實糾正格）'!A39</f>
         <v/>
       </c>
       <c r="I39">
-        <f>'第三人評分（限事實糾正格）'!C39</f>
+        <f>'Coder 3評分（限事實糾正格）'!C39</f>
         <v/>
       </c>
       <c r="J39">
-        <f>IFERROR(XLOOKUP(H39,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H39,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="H40">
-        <f>'第三人評分（限事實糾正格）'!A40</f>
+        <f>'Coder 3評分（限事實糾正格）'!A40</f>
         <v/>
       </c>
       <c r="I40">
-        <f>'第三人評分（限事實糾正格）'!C40</f>
+        <f>'Coder 3評分（限事實糾正格）'!C40</f>
         <v/>
       </c>
       <c r="J40">
-        <f>IFERROR(XLOOKUP(H40,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H40,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="H41">
-        <f>'第三人評分（限事實糾正格）'!A41</f>
+        <f>'Coder 3評分（限事實糾正格）'!A41</f>
         <v/>
       </c>
       <c r="I41">
-        <f>'第三人評分（限事實糾正格）'!C41</f>
+        <f>'Coder 3評分（限事實糾正格）'!C41</f>
         <v/>
       </c>
       <c r="J41">
-        <f>IFERROR(XLOOKUP(H41,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H41,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="H42">
-        <f>'第三人評分（限事實糾正格）'!A42</f>
+        <f>'Coder 3評分（限事實糾正格）'!A42</f>
         <v/>
       </c>
       <c r="I42">
-        <f>'第三人評分（限事實糾正格）'!C42</f>
+        <f>'Coder 3評分（限事實糾正格）'!C42</f>
         <v/>
       </c>
       <c r="J42">
-        <f>IFERROR(XLOOKUP(H42,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H42,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="H43">
-        <f>'第三人評分（限事實糾正格）'!A43</f>
+        <f>'Coder 3評分（限事實糾正格）'!A43</f>
         <v/>
       </c>
       <c r="I43">
-        <f>'第三人評分（限事實糾正格）'!C43</f>
+        <f>'Coder 3評分（限事實糾正格）'!C43</f>
         <v/>
       </c>
       <c r="J43">
-        <f>IFERROR(XLOOKUP(H43,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H43,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="H44">
-        <f>'第三人評分（限事實糾正格）'!A44</f>
+        <f>'Coder 3評分（限事實糾正格）'!A44</f>
         <v/>
       </c>
       <c r="I44">
-        <f>'第三人評分（限事實糾正格）'!C44</f>
+        <f>'Coder 3評分（限事實糾正格）'!C44</f>
         <v/>
       </c>
       <c r="J44">
-        <f>IFERROR(XLOOKUP(H44,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H44,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="H45">
-        <f>'第三人評分（限事實糾正格）'!A45</f>
+        <f>'Coder 3評分（限事實糾正格）'!A45</f>
         <v/>
       </c>
       <c r="I45">
-        <f>'第三人評分（限事實糾正格）'!C45</f>
+        <f>'Coder 3評分（限事實糾正格）'!C45</f>
         <v/>
       </c>
       <c r="J45">
-        <f>IFERROR(XLOOKUP(H45,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H45,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="H46">
-        <f>'第三人評分（限事實糾正格）'!A46</f>
+        <f>'Coder 3評分（限事實糾正格）'!A46</f>
         <v/>
       </c>
       <c r="I46">
-        <f>'第三人評分（限事實糾正格）'!C46</f>
+        <f>'Coder 3評分（限事實糾正格）'!C46</f>
         <v/>
       </c>
       <c r="J46">
-        <f>IFERROR(XLOOKUP(H46,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H46,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="H47">
-        <f>'第三人評分（限事實糾正格）'!A47</f>
+        <f>'Coder 3評分（限事實糾正格）'!A47</f>
         <v/>
       </c>
       <c r="I47">
-        <f>'第三人評分（限事實糾正格）'!C47</f>
+        <f>'Coder 3評分（限事實糾正格）'!C47</f>
         <v/>
       </c>
       <c r="J47">
-        <f>IFERROR(XLOOKUP(H47,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H47,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="H48">
-        <f>'第三人評分（限事實糾正格）'!A48</f>
+        <f>'Coder 3評分（限事實糾正格）'!A48</f>
         <v/>
       </c>
       <c r="I48">
-        <f>'第三人評分（限事實糾正格）'!C48</f>
+        <f>'Coder 3評分（限事實糾正格）'!C48</f>
         <v/>
       </c>
       <c r="J48">
-        <f>IFERROR(XLOOKUP(H48,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H48,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="H49">
-        <f>'第三人評分（限事實糾正格）'!A49</f>
+        <f>'Coder 3評分（限事實糾正格）'!A49</f>
         <v/>
       </c>
       <c r="I49">
-        <f>'第三人評分（限事實糾正格）'!C49</f>
+        <f>'Coder 3評分（限事實糾正格）'!C49</f>
         <v/>
       </c>
       <c r="J49">
-        <f>IFERROR(XLOOKUP(H49,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H49,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="H50">
-        <f>'第三人評分（限事實糾正格）'!A50</f>
+        <f>'Coder 3評分（限事實糾正格）'!A50</f>
         <v/>
       </c>
       <c r="I50">
-        <f>'第三人評分（限事實糾正格）'!C50</f>
+        <f>'Coder 3評分（限事實糾正格）'!C50</f>
         <v/>
       </c>
       <c r="J50">
-        <f>IFERROR(XLOOKUP(H50,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H50,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="H51">
-        <f>'第三人評分（限事實糾正格）'!A51</f>
+        <f>'Coder 3評分（限事實糾正格）'!A51</f>
         <v/>
       </c>
       <c r="I51">
-        <f>'第三人評分（限事實糾正格）'!C51</f>
+        <f>'Coder 3評分（限事實糾正格）'!C51</f>
         <v/>
       </c>
       <c r="J51">
-        <f>IFERROR(XLOOKUP(H51,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H51,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="H52">
-        <f>'第三人評分（限事實糾正格）'!A52</f>
+        <f>'Coder 3評分（限事實糾正格）'!A52</f>
         <v/>
       </c>
       <c r="I52">
-        <f>'第三人評分（限事實糾正格）'!C52</f>
+        <f>'Coder 3評分（限事實糾正格）'!C52</f>
         <v/>
       </c>
       <c r="J52">
-        <f>IFERROR(XLOOKUP(H52,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H52,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="H53">
-        <f>'第三人評分（限事實糾正格）'!A53</f>
+        <f>'Coder 3評分（限事實糾正格）'!A53</f>
         <v/>
       </c>
       <c r="I53">
-        <f>'第三人評分（限事實糾正格）'!C53</f>
+        <f>'Coder 3評分（限事實糾正格）'!C53</f>
         <v/>
       </c>
       <c r="J53">
-        <f>IFERROR(XLOOKUP(H53,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H53,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="H54">
-        <f>'第三人評分（限事實糾正格）'!A54</f>
+        <f>'Coder 3評分（限事實糾正格）'!A54</f>
         <v/>
       </c>
       <c r="I54">
-        <f>'第三人評分（限事實糾正格）'!C54</f>
+        <f>'Coder 3評分（限事實糾正格）'!C54</f>
         <v/>
       </c>
       <c r="J54">
-        <f>IFERROR(XLOOKUP(H54,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H54,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="H55">
-        <f>'第三人評分（限事實糾正格）'!A55</f>
+        <f>'Coder 3評分（限事實糾正格）'!A55</f>
         <v/>
       </c>
       <c r="I55">
-        <f>'第三人評分（限事實糾正格）'!C55</f>
+        <f>'Coder 3評分（限事實糾正格）'!C55</f>
         <v/>
       </c>
       <c r="J55">
-        <f>IFERROR(XLOOKUP(H55,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H55,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="H56">
-        <f>'第三人評分（限事實糾正格）'!A56</f>
+        <f>'Coder 3評分（限事實糾正格）'!A56</f>
         <v/>
       </c>
       <c r="I56">
-        <f>'第三人評分（限事實糾正格）'!C56</f>
+        <f>'Coder 3評分（限事實糾正格）'!C56</f>
         <v/>
       </c>
       <c r="J56">
-        <f>IFERROR(XLOOKUP(H56,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H56,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="H57">
-        <f>'第三人評分（限事實糾正格）'!A57</f>
+        <f>'Coder 3評分（限事實糾正格）'!A57</f>
         <v/>
       </c>
       <c r="I57">
-        <f>'第三人評分（限事實糾正格）'!C57</f>
+        <f>'Coder 3評分（限事實糾正格）'!C57</f>
         <v/>
       </c>
       <c r="J57">
-        <f>IFERROR(XLOOKUP(H57,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H57,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="H58">
-        <f>'第三人評分（限事實糾正格）'!A58</f>
+        <f>'Coder 3評分（限事實糾正格）'!A58</f>
         <v/>
       </c>
       <c r="I58">
-        <f>'第三人評分（限事實糾正格）'!C58</f>
+        <f>'Coder 3評分（限事實糾正格）'!C58</f>
         <v/>
       </c>
       <c r="J58">
-        <f>IFERROR(XLOOKUP(H58,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H58,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="H59">
-        <f>'第三人評分（限事實糾正格）'!A59</f>
+        <f>'Coder 3評分（限事實糾正格）'!A59</f>
         <v/>
       </c>
       <c r="I59">
-        <f>'第三人評分（限事實糾正格）'!C59</f>
+        <f>'Coder 3評分（限事實糾正格）'!C59</f>
         <v/>
       </c>
       <c r="J59">
-        <f>IFERROR(XLOOKUP(H59,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H59,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="H60">
-        <f>'第三人評分（限事實糾正格）'!A60</f>
+        <f>'Coder 3評分（限事實糾正格）'!A60</f>
         <v/>
       </c>
       <c r="I60">
-        <f>'第三人評分（限事實糾正格）'!C60</f>
+        <f>'Coder 3評分（限事實糾正格）'!C60</f>
         <v/>
       </c>
       <c r="J60">
-        <f>IFERROR(XLOOKUP(H60,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H60,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="H61">
-        <f>'第三人評分（限事實糾正格）'!A61</f>
+        <f>'Coder 3評分（限事實糾正格）'!A61</f>
         <v/>
       </c>
       <c r="I61">
-        <f>'第三人評分（限事實糾正格）'!C61</f>
+        <f>'Coder 3評分（限事實糾正格）'!C61</f>
         <v/>
       </c>
       <c r="J61">
-        <f>IFERROR(XLOOKUP(H61,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H61,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="H62">
-        <f>'第三人評分（限事實糾正格）'!A62</f>
+        <f>'Coder 3評分（限事實糾正格）'!A62</f>
         <v/>
       </c>
       <c r="I62">
-        <f>'第三人評分（限事實糾正格）'!C62</f>
+        <f>'Coder 3評分（限事實糾正格）'!C62</f>
         <v/>
       </c>
       <c r="J62">
-        <f>IFERROR(XLOOKUP(H62,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H62,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="H63">
-        <f>'第三人評分（限事實糾正格）'!A63</f>
+        <f>'Coder 3評分（限事實糾正格）'!A63</f>
         <v/>
       </c>
       <c r="I63">
-        <f>'第三人評分（限事實糾正格）'!C63</f>
+        <f>'Coder 3評分（限事實糾正格）'!C63</f>
         <v/>
       </c>
       <c r="J63">
-        <f>IFERROR(XLOOKUP(H63,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H63,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="H64">
-        <f>'第三人評分（限事實糾正格）'!A64</f>
+        <f>'Coder 3評分（限事實糾正格）'!A64</f>
         <v/>
       </c>
       <c r="I64">
-        <f>'第三人評分（限事實糾正格）'!C64</f>
+        <f>'Coder 3評分（限事實糾正格）'!C64</f>
         <v/>
       </c>
       <c r="J64">
-        <f>IFERROR(XLOOKUP(H64,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H64,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="H65">
-        <f>'第三人評分（限事實糾正格）'!A65</f>
+        <f>'Coder 3評分（限事實糾正格）'!A65</f>
         <v/>
       </c>
       <c r="I65">
-        <f>'第三人評分（限事實糾正格）'!C65</f>
+        <f>'Coder 3評分（限事實糾正格）'!C65</f>
         <v/>
       </c>
       <c r="J65">
-        <f>IFERROR(XLOOKUP(H65,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H65,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="H66">
-        <f>'第三人評分（限事實糾正格）'!A66</f>
+        <f>'Coder 3評分（限事實糾正格）'!A66</f>
         <v/>
       </c>
       <c r="I66">
-        <f>'第三人評分（限事實糾正格）'!C66</f>
+        <f>'Coder 3評分（限事實糾正格）'!C66</f>
         <v/>
       </c>
       <c r="J66">
-        <f>IFERROR(XLOOKUP(H66,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H66,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="H67">
-        <f>'第三人評分（限事實糾正格）'!A67</f>
+        <f>'Coder 3評分（限事實糾正格）'!A67</f>
         <v/>
       </c>
       <c r="I67">
-        <f>'第三人評分（限事實糾正格）'!C67</f>
+        <f>'Coder 3評分（限事實糾正格）'!C67</f>
         <v/>
       </c>
       <c r="J67">
-        <f>IFERROR(XLOOKUP(H67,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H67,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="H68">
-        <f>'第三人評分（限事實糾正格）'!A68</f>
+        <f>'Coder 3評分（限事實糾正格）'!A68</f>
         <v/>
       </c>
       <c r="I68">
-        <f>'第三人評分（限事實糾正格）'!C68</f>
+        <f>'Coder 3評分（限事實糾正格）'!C68</f>
         <v/>
       </c>
       <c r="J68">
-        <f>IFERROR(XLOOKUP(H68,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H68,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="H69">
-        <f>'第三人評分（限事實糾正格）'!A69</f>
+        <f>'Coder 3評分（限事實糾正格）'!A69</f>
         <v/>
       </c>
       <c r="I69">
-        <f>'第三人評分（限事實糾正格）'!C69</f>
+        <f>'Coder 3評分（限事實糾正格）'!C69</f>
         <v/>
       </c>
       <c r="J69">
-        <f>IFERROR(XLOOKUP(H69,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H69,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="H70">
-        <f>'第三人評分（限事實糾正格）'!A70</f>
+        <f>'Coder 3評分（限事實糾正格）'!A70</f>
         <v/>
       </c>
       <c r="I70">
-        <f>'第三人評分（限事實糾正格）'!C70</f>
+        <f>'Coder 3評分（限事實糾正格）'!C70</f>
         <v/>
       </c>
       <c r="J70">
-        <f>IFERROR(XLOOKUP(H70,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H70,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="H71">
-        <f>'第三人評分（限事實糾正格）'!A71</f>
+        <f>'Coder 3評分（限事實糾正格）'!A71</f>
         <v/>
       </c>
       <c r="I71">
-        <f>'第三人評分（限事實糾正格）'!C71</f>
+        <f>'Coder 3評分（限事實糾正格）'!C71</f>
         <v/>
       </c>
       <c r="J71">
-        <f>IFERROR(XLOOKUP(H71,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H71,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="H72">
-        <f>'第三人評分（限事實糾正格）'!A72</f>
+        <f>'Coder 3評分（限事實糾正格）'!A72</f>
         <v/>
       </c>
       <c r="I72">
-        <f>'第三人評分（限事實糾正格）'!C72</f>
+        <f>'Coder 3評分（限事實糾正格）'!C72</f>
         <v/>
       </c>
       <c r="J72">
-        <f>IFERROR(XLOOKUP(H72,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H72,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="H73">
-        <f>'第三人評分（限事實糾正格）'!A73</f>
+        <f>'Coder 3評分（限事實糾正格）'!A73</f>
         <v/>
       </c>
       <c r="I73">
-        <f>'第三人評分（限事實糾正格）'!C73</f>
+        <f>'Coder 3評分（限事實糾正格）'!C73</f>
         <v/>
       </c>
       <c r="J73">
-        <f>IFERROR(XLOOKUP(H73,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H73,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="H74">
-        <f>'第三人評分（限事實糾正格）'!A74</f>
+        <f>'Coder 3評分（限事實糾正格）'!A74</f>
         <v/>
       </c>
       <c r="I74">
-        <f>'第三人評分（限事實糾正格）'!C74</f>
+        <f>'Coder 3評分（限事實糾正格）'!C74</f>
         <v/>
       </c>
       <c r="J74">
-        <f>IFERROR(XLOOKUP(H74,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H74,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="H75">
-        <f>'第三人評分（限事實糾正格）'!A75</f>
+        <f>'Coder 3評分（限事實糾正格）'!A75</f>
         <v/>
       </c>
       <c r="I75">
-        <f>'第三人評分（限事實糾正格）'!C75</f>
+        <f>'Coder 3評分（限事實糾正格）'!C75</f>
         <v/>
       </c>
       <c r="J75">
-        <f>IFERROR(XLOOKUP(H75,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H75,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="H76">
-        <f>'第三人評分（限事實糾正格）'!A76</f>
+        <f>'Coder 3評分（限事實糾正格）'!A76</f>
         <v/>
       </c>
       <c r="I76">
-        <f>'第三人評分（限事實糾正格）'!C76</f>
+        <f>'Coder 3評分（限事實糾正格）'!C76</f>
         <v/>
       </c>
       <c r="J76">
-        <f>IFERROR(XLOOKUP(H76,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H76,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="H77">
-        <f>'第三人評分（限事實糾正格）'!A77</f>
+        <f>'Coder 3評分（限事實糾正格）'!A77</f>
         <v/>
       </c>
       <c r="I77">
-        <f>'第三人評分（限事實糾正格）'!C77</f>
+        <f>'Coder 3評分（限事實糾正格）'!C77</f>
         <v/>
       </c>
       <c r="J77">
-        <f>IFERROR(XLOOKUP(H77,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H77,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="H78">
-        <f>'第三人評分（限事實糾正格）'!A78</f>
+        <f>'Coder 3評分（限事實糾正格）'!A78</f>
         <v/>
       </c>
       <c r="I78">
-        <f>'第三人評分（限事實糾正格）'!C78</f>
+        <f>'Coder 3評分（限事實糾正格）'!C78</f>
         <v/>
       </c>
       <c r="J78">
-        <f>IFERROR(XLOOKUP(H78,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H78,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="H79">
-        <f>'第三人評分（限事實糾正格）'!A79</f>
+        <f>'Coder 3評分（限事實糾正格）'!A79</f>
         <v/>
       </c>
       <c r="I79">
-        <f>'第三人評分（限事實糾正格）'!C79</f>
+        <f>'Coder 3評分（限事實糾正格）'!C79</f>
         <v/>
       </c>
       <c r="J79">
-        <f>IFERROR(XLOOKUP(H79,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H79,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="H80">
-        <f>'第三人評分（限事實糾正格）'!A80</f>
+        <f>'Coder 3評分（限事實糾正格）'!A80</f>
         <v/>
       </c>
       <c r="I80">
-        <f>'第三人評分（限事實糾正格）'!C80</f>
+        <f>'Coder 3評分（限事實糾正格）'!C80</f>
         <v/>
       </c>
       <c r="J80">
-        <f>IFERROR(XLOOKUP(H80,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H80,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="H81">
-        <f>'第三人評分（限事實糾正格）'!A81</f>
+        <f>'Coder 3評分（限事實糾正格）'!A81</f>
         <v/>
       </c>
       <c r="I81">
-        <f>'第三人評分（限事實糾正格）'!C81</f>
+        <f>'Coder 3評分（限事實糾正格）'!C81</f>
         <v/>
       </c>
       <c r="J81">
-        <f>IFERROR(XLOOKUP(H81,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H81,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="H82">
-        <f>'第三人評分（限事實糾正格）'!A82</f>
+        <f>'Coder 3評分（限事實糾正格）'!A82</f>
         <v/>
       </c>
       <c r="I82">
-        <f>'第三人評分（限事實糾正格）'!C82</f>
+        <f>'Coder 3評分（限事實糾正格）'!C82</f>
         <v/>
       </c>
       <c r="J82">
-        <f>IFERROR(XLOOKUP(H82,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H82,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="H83">
-        <f>'第三人評分（限事實糾正格）'!A83</f>
+        <f>'Coder 3評分（限事實糾正格）'!A83</f>
         <v/>
       </c>
       <c r="I83">
-        <f>'第三人評分（限事實糾正格）'!C83</f>
+        <f>'Coder 3評分（限事實糾正格）'!C83</f>
         <v/>
       </c>
       <c r="J83">
-        <f>IFERROR(XLOOKUP(H83,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H83,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="H84">
-        <f>'第三人評分（限事實糾正格）'!A84</f>
+        <f>'Coder 3評分（限事實糾正格）'!A84</f>
         <v/>
       </c>
       <c r="I84">
-        <f>'第三人評分（限事實糾正格）'!C84</f>
+        <f>'Coder 3評分（限事實糾正格）'!C84</f>
         <v/>
       </c>
       <c r="J84">
-        <f>IFERROR(XLOOKUP(H84,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H84,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="H85">
-        <f>'第三人評分（限事實糾正格）'!A85</f>
+        <f>'Coder 3評分（限事實糾正格）'!A85</f>
         <v/>
       </c>
       <c r="I85">
-        <f>'第三人評分（限事實糾正格）'!C85</f>
+        <f>'Coder 3評分（限事實糾正格）'!C85</f>
         <v/>
       </c>
       <c r="J85">
-        <f>IFERROR(XLOOKUP(H85,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H85,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="H86">
-        <f>'第三人評分（限事實糾正格）'!A86</f>
+        <f>'Coder 3評分（限事實糾正格）'!A86</f>
         <v/>
       </c>
       <c r="I86">
-        <f>'第三人評分（限事實糾正格）'!C86</f>
+        <f>'Coder 3評分（限事實糾正格）'!C86</f>
         <v/>
       </c>
       <c r="J86">
-        <f>IFERROR(XLOOKUP(H86,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H86,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="H87">
-        <f>'第三人評分（限事實糾正格）'!A87</f>
+        <f>'Coder 3評分（限事實糾正格）'!A87</f>
         <v/>
       </c>
       <c r="I87">
-        <f>'第三人評分（限事實糾正格）'!C87</f>
+        <f>'Coder 3評分（限事實糾正格）'!C87</f>
         <v/>
       </c>
       <c r="J87">
-        <f>IFERROR(XLOOKUP(H87,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H87,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="H88">
-        <f>'第三人評分（限事實糾正格）'!A88</f>
+        <f>'Coder 3評分（限事實糾正格）'!A88</f>
         <v/>
       </c>
       <c r="I88">
-        <f>'第三人評分（限事實糾正格）'!C88</f>
+        <f>'Coder 3評分（限事實糾正格）'!C88</f>
         <v/>
       </c>
       <c r="J88">
-        <f>IFERROR(XLOOKUP(H88,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H88,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="H89">
-        <f>'第三人評分（限事實糾正格）'!A89</f>
+        <f>'Coder 3評分（限事實糾正格）'!A89</f>
         <v/>
       </c>
       <c r="I89">
-        <f>'第三人評分（限事實糾正格）'!C89</f>
+        <f>'Coder 3評分（限事實糾正格）'!C89</f>
         <v/>
       </c>
       <c r="J89">
-        <f>IFERROR(XLOOKUP(H89,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H89,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="H90">
-        <f>'第三人評分（限事實糾正格）'!A90</f>
+        <f>'Coder 3評分（限事實糾正格）'!A90</f>
         <v/>
       </c>
       <c r="I90">
-        <f>'第三人評分（限事實糾正格）'!C90</f>
+        <f>'Coder 3評分（限事實糾正格）'!C90</f>
         <v/>
       </c>
       <c r="J90">
-        <f>IFERROR(XLOOKUP(H90,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H90,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="H91">
-        <f>'第三人評分（限事實糾正格）'!A91</f>
+        <f>'Coder 3評分（限事實糾正格）'!A91</f>
         <v/>
       </c>
       <c r="I91">
-        <f>'第三人評分（限事實糾正格）'!C91</f>
+        <f>'Coder 3評分（限事實糾正格）'!C91</f>
         <v/>
       </c>
       <c r="J91">
-        <f>IFERROR(XLOOKUP(H91,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H91,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="92">
       <c r="H92">
-        <f>'第三人評分（限事實糾正格）'!A92</f>
+        <f>'Coder 3評分（限事實糾正格）'!A92</f>
         <v/>
       </c>
       <c r="I92">
-        <f>'第三人評分（限事實糾正格）'!C92</f>
+        <f>'Coder 3評分（限事實糾正格）'!C92</f>
         <v/>
       </c>
       <c r="J92">
-        <f>IFERROR(XLOOKUP(H92,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H92,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="93">
       <c r="H93">
-        <f>'第三人評分（限事實糾正格）'!A93</f>
+        <f>'Coder 3評分（限事實糾正格）'!A93</f>
         <v/>
       </c>
       <c r="I93">
-        <f>'第三人評分（限事實糾正格）'!C93</f>
+        <f>'Coder 3評分（限事實糾正格）'!C93</f>
         <v/>
       </c>
       <c r="J93">
-        <f>IFERROR(XLOOKUP(H93,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H93,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="94">
       <c r="H94">
-        <f>'第三人評分（限事實糾正格）'!A94</f>
+        <f>'Coder 3評分（限事實糾正格）'!A94</f>
         <v/>
       </c>
       <c r="I94">
-        <f>'第三人評分（限事實糾正格）'!C94</f>
+        <f>'Coder 3評分（限事實糾正格）'!C94</f>
         <v/>
       </c>
       <c r="J94">
-        <f>IFERROR(XLOOKUP(H94,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H94,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="H95">
-        <f>'第三人評分（限事實糾正格）'!A95</f>
+        <f>'Coder 3評分（限事實糾正格）'!A95</f>
         <v/>
       </c>
       <c r="I95">
-        <f>'第三人評分（限事實糾正格）'!C95</f>
+        <f>'Coder 3評分（限事實糾正格）'!C95</f>
         <v/>
       </c>
       <c r="J95">
-        <f>IFERROR(XLOOKUP(H95,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H95,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="96">
       <c r="H96">
-        <f>'第三人評分（限事實糾正格）'!A96</f>
+        <f>'Coder 3評分（限事實糾正格）'!A96</f>
         <v/>
       </c>
       <c r="I96">
-        <f>'第三人評分（限事實糾正格）'!C96</f>
+        <f>'Coder 3評分（限事實糾正格）'!C96</f>
         <v/>
       </c>
       <c r="J96">
-        <f>IFERROR(XLOOKUP(H96,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H96,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="97">
       <c r="H97">
-        <f>'第三人評分（限事實糾正格）'!A97</f>
+        <f>'Coder 3評分（限事實糾正格）'!A97</f>
         <v/>
       </c>
       <c r="I97">
-        <f>'第三人評分（限事實糾正格）'!C97</f>
+        <f>'Coder 3評分（限事實糾正格）'!C97</f>
         <v/>
       </c>
       <c r="J97">
-        <f>IFERROR(XLOOKUP(H97,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H97,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="98">
       <c r="H98">
-        <f>'第三人評分（限事實糾正格）'!A98</f>
+        <f>'Coder 3評分（限事實糾正格）'!A98</f>
         <v/>
       </c>
       <c r="I98">
-        <f>'第三人評分（限事實糾正格）'!C98</f>
+        <f>'Coder 3評分（限事實糾正格）'!C98</f>
         <v/>
       </c>
       <c r="J98">
-        <f>IFERROR(XLOOKUP(H98,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H98,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="99">
       <c r="H99">
-        <f>'第三人評分（限事實糾正格）'!A99</f>
+        <f>'Coder 3評分（限事實糾正格）'!A99</f>
         <v/>
       </c>
       <c r="I99">
-        <f>'第三人評分（限事實糾正格）'!C99</f>
+        <f>'Coder 3評分（限事實糾正格）'!C99</f>
         <v/>
       </c>
       <c r="J99">
-        <f>IFERROR(XLOOKUP(H99,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H99,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="100">
       <c r="H100">
-        <f>'第三人評分（限事實糾正格）'!A100</f>
+        <f>'Coder 3評分（限事實糾正格）'!A100</f>
         <v/>
       </c>
       <c r="I100">
-        <f>'第三人評分（限事實糾正格）'!C100</f>
+        <f>'Coder 3評分（限事實糾正格）'!C100</f>
         <v/>
       </c>
       <c r="J100">
-        <f>IFERROR(XLOOKUP(H100,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H100,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="101">
       <c r="H101">
-        <f>'第三人評分（限事實糾正格）'!A101</f>
+        <f>'Coder 3評分（限事實糾正格）'!A101</f>
         <v/>
       </c>
       <c r="I101">
-        <f>'第三人評分（限事實糾正格）'!C101</f>
+        <f>'Coder 3評分（限事實糾正格）'!C101</f>
         <v/>
       </c>
       <c r="J101">
-        <f>IFERROR(XLOOKUP(H101,'地理老師評分'!$A$2:$A$101,'地理老師評分'!$R$2:$R$101,""),"")</f>
+        <f>IFERROR(XLOOKUP(H101,'Coder 2評分'!$A$2:$A$101,'Coder 2評分'!$R$2:$R$101,""),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>